<commit_message>
Update MLP Excel tutorial
</commit_message>
<xml_diff>
--- a/4. Supervised Learning (modeling and evaluation)/biases_layer1.xlsx
+++ b/4. Supervised Learning (modeling and evaluation)/biases_layer1.xlsx
@@ -435,502 +435,502 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.2111082486469878</v>
+        <v>-0.1276842812615124</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.06414997389744802</v>
+        <v>-0.07936059193498547</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.09210160235946625</v>
+        <v>-0.2191401007507529</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>-0.1821142619838667</v>
+        <v>0.2323022538187379</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>-0.02559871004068377</v>
+        <v>-0.0001651436349512851</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>-0.1815075241531962</v>
+        <v>0.03996903923528149</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>-0.00735726148463216</v>
+        <v>-0.1631412921817638</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>-0.2218523015610998</v>
+        <v>-0.03246824190568413</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>-0.1192217867025647</v>
+        <v>0.00593851318482802</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0.2011754710794841</v>
+        <v>-0.01923236583885896</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>0.1344785409531422</v>
+        <v>-0.1451586196307538</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>-0.1638994855601357</v>
+        <v>-0.06112621777209485</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>-0.04484724571086613</v>
+        <v>-0.1400190261446417</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>-0.03661703203662606</v>
+        <v>-0.2049109635638666</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>-0.2051552731168239</v>
+        <v>0.09584253425925383</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>-0.1255791606535179</v>
+        <v>0.2438219069452465</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>-0.002493646725150237</v>
+        <v>0.1133788838806436</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>-0.07479803411128776</v>
+        <v>0.01511528294839182</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>-0.1902967474699822</v>
+        <v>-0.01471064984087447</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>0.1582600891701293</v>
+        <v>0.08138129492162512</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>0.171804741552715</v>
+        <v>-0.2161891230489796</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>-0.2121795196643959</v>
+        <v>-0.128921416578491</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>-0.06220735840516253</v>
+        <v>0.03287608161710818</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>0.08440260671209895</v>
+        <v>0.1722026772008274</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>0.1728045843169319</v>
+        <v>0.171157987511577</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>-0.00664776945763948</v>
+        <v>0.1210741150174491</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>0.1389095034450491</v>
+        <v>-0.2486153714049599</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>0.02792140380329701</v>
+        <v>0.002749674527381674</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>0.1894247832423779</v>
+        <v>-0.07983958159245555</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>0.219937292257647</v>
+        <v>-0.176981174853441</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>0.1954903901023159</v>
+        <v>-0.06656491589745821</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>0.009164476711680766</v>
+        <v>-0.1713717260834565</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>0.2360742116548003</v>
+        <v>0.02280356049433908</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>0.03020805064337876</v>
+        <v>-0.113002907051043</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>0.1431068484809864</v>
+        <v>0.05453873941709994</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>-0.1458632878776443</v>
+        <v>0.01882532422765058</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>-0.1217440109216782</v>
+        <v>0.09511563191284783</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>0.2292710231352372</v>
+        <v>0.1082273909129281</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>-0.06553417229359523</v>
+        <v>0.1584213087730452</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>0.2021485626181914</v>
+        <v>0.2497454730263628</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>-0.02829768313391136</v>
+        <v>-0.2087232110563569</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>0.2508191901782723</v>
+        <v>-0.221779287815745</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>0.2180886771814237</v>
+        <v>-0.09287876761608339</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>-0.1540810582941617</v>
+        <v>-0.2031576307822749</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>-0.1772179003133222</v>
+        <v>0.214943740823647</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>0.09586944393956069</v>
+        <v>0.1786991402117721</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>-0.02977707576239381</v>
+        <v>0.08016435460237566</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>0.141942009416966</v>
+        <v>0.09473759602481741</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>0.1478898616533398</v>
+        <v>-0.08100131187263071</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>0.2053831412627123</v>
+        <v>0.1835332282499585</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>0.1124964792596113</v>
+        <v>-0.1861042699811559</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>-0.0945651815034305</v>
+        <v>0.09267848531796143</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>0.05767299946122879</v>
+        <v>-0.06774420438464297</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>-0.05348301885733167</v>
+        <v>0.1906710589750211</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>-0.05909499810137565</v>
+        <v>-0.1230786763913912</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>0.08461505097730632</v>
+        <v>0.06852138385752231</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>-0.03875436258092062</v>
+        <v>-0.2316711355965107</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>0.1127038487004757</v>
+        <v>0.09265978972187133</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>-0.1505862148432725</v>
+        <v>0.1138954989585571</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>0.2122771127686186</v>
+        <v>0.1856911003581369</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>-0.05793621661417598</v>
+        <v>-0.06589353077269733</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>-0.07446942702575773</v>
+        <v>-0.2238046011970296</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>-0.1352255563765146</v>
+        <v>-0.1780113546539159</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>-0.1075150677173567</v>
+        <v>0.1778384045672716</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>0.1501243581209412</v>
+        <v>0.06085968904320999</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>-0.04752829357193275</v>
+        <v>-0.2161155394695577</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>0.2065915401545691</v>
+        <v>0.1997794032346849</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>0.002838216605631509</v>
+        <v>0.1897035434258542</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>-0.2439352723541783</v>
+        <v>0.02941721211965852</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>-0.1105502418338554</v>
+        <v>0.09774542411774004</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>0.1337822892363713</v>
+        <v>0.2311401671616378</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>-0.1436915596966477</v>
+        <v>0.001219975979007298</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>0.1818743434193317</v>
+        <v>-0.1334290723592081</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>0.008554307059682976</v>
+        <v>0.1830021674028805</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>-0.0535795652181268</v>
+        <v>0.07162082011838095</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>0.153347277294905</v>
+        <v>-0.1601101109665211</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>-0.03040765280462301</v>
+        <v>-0.2297357677947958</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>-0.1899108518844683</v>
+        <v>0.1037664654845489</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>0.2175447521813219</v>
+        <v>0.07552250738582816</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>0.01245270987472315</v>
+        <v>-0.231665456086941</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>0.09135314999335725</v>
+        <v>-0.2020429820912898</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>0.1109453164881298</v>
+        <v>-0.09707590426964005</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>-0.04796391348036017</v>
+        <v>-0.035147983770233</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>0.02441995615995809</v>
+        <v>0.066553184776954</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>0.09605081379987329</v>
+        <v>-0.02769102741440754</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>0.004435251347976899</v>
+        <v>-0.1599042362243941</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>0.079741758164335</v>
+        <v>0.2298740244589949</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>-0.02421274407724677</v>
+        <v>-0.1091663540194024</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>0.0649062467635635</v>
+        <v>-0.1580115760197517</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>0.1654182840096088</v>
+        <v>0.219160109514121</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>0.1939492266571343</v>
+        <v>-0.1838508806342038</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>0.1691781805994081</v>
+        <v>0.2291767940961008</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>-0.1699384139062234</v>
+        <v>-0.05317284465409905</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>-0.0318941217878279</v>
+        <v>-0.08356216039643237</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>0.01870596031791316</v>
+        <v>0.1785550703945179</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>-0.2213712975348801</v>
+        <v>-0.1874685790414486</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>-0.1436170066650786</v>
+        <v>-0.1132884208034727</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>0.0916636499712417</v>
+        <v>0.04669586727591851</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>0.09542025782203931</v>
+        <v>-0.1501056248283371</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>-0.03490038349273577</v>
+        <v>-0.006182075291396754</v>
       </c>
     </row>
   </sheetData>

</xml_diff>